<commit_message>
Update LMO HULU LUC recaps from corrected SimaPro export
</commit_message>
<xml_diff>
--- a/Rekap_LCI_LMO.xlsx
+++ b/Rekap_LCI_LMO.xlsx
@@ -6,12 +6,14 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="14400" windowHeight="15750" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LCI INTI LMO" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LCI UT LMO" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LCI HULU LMO" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LCI INTI LMO" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LCI UT LMO" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'LCI INTI LMO'!$B$2:$I$87</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'LCI UT LMO'!$B$2:$I$82</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'LCI HULU LMO'!$B$2:$I$69</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'LCI INTI LMO'!$B$2:$I$87</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'LCI UT LMO'!$B$2:$I$82</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -210,12 +212,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
+        <fgColor rgb="00F3F7F9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F3F7F9"/>
+        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -962,6 +964,2206 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
+  <dimension ref="B2:I69"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="39" customWidth="1" min="3" max="3"/>
+    <col width="70" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="25" customHeight="1">
+      <c r="B2" s="33" t="inlineStr">
+        <is>
+          <t>HASIL ANALISIS ISU PENTING BERDASARKAN INVENTORY PRODUK — HULU LMO
+Kontribusi Pareto ≥80% per kategori dampak</t>
+        </is>
+      </c>
+      <c r="C2" s="34" t="n"/>
+      <c r="D2" s="34" t="n"/>
+      <c r="E2" s="34" t="n"/>
+      <c r="F2" s="34" t="n"/>
+      <c r="G2" s="34" t="n"/>
+      <c r="H2" s="34" t="n"/>
+      <c r="I2" s="35" t="n"/>
+    </row>
+    <row r="3" ht="25" customHeight="1">
+      <c r="B3" s="36" t="n"/>
+      <c r="C3" s="37" t="n"/>
+      <c r="D3" s="37" t="n"/>
+      <c r="E3" s="37" t="n"/>
+      <c r="F3" s="37" t="n"/>
+      <c r="G3" s="37" t="n"/>
+      <c r="H3" s="37" t="n"/>
+      <c r="I3" s="38" t="n"/>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="B5" s="22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C5" s="22" t="inlineStr">
+        <is>
+          <t>Kategori Dampak</t>
+        </is>
+      </c>
+      <c r="D5" s="22" t="inlineStr">
+        <is>
+          <t>Unit proses / proses terkait (bukan asal inventori)*</t>
+        </is>
+      </c>
+      <c r="E5" s="22" t="inlineStr">
+        <is>
+          <t>Inventori / substansi penyebab</t>
+        </is>
+      </c>
+      <c r="F5" s="22" t="inlineStr">
+        <is>
+          <t>Nilai dampak</t>
+        </is>
+      </c>
+      <c r="G5" s="22" t="inlineStr">
+        <is>
+          <t>Satuan</t>
+        </is>
+      </c>
+      <c r="H5" s="22" t="inlineStr">
+        <is>
+          <t>Kontribusi bertanda</t>
+        </is>
+      </c>
+      <c r="I5" s="22" t="inlineStr">
+        <is>
+          <t>Kumulatif arah neto</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="B6" s="39" t="n"/>
+      <c r="C6" s="39" t="n"/>
+      <c r="D6" s="39" t="n"/>
+      <c r="E6" s="39" t="n"/>
+      <c r="F6" s="39" t="n"/>
+      <c r="G6" s="39" t="n"/>
+      <c r="H6" s="39" t="n"/>
+      <c r="I6" s="39" t="n"/>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="B7" s="40" t="n"/>
+      <c r="C7" s="40" t="n"/>
+      <c r="D7" s="40" t="n"/>
+      <c r="E7" s="40" t="n"/>
+      <c r="F7" s="40" t="n"/>
+      <c r="G7" s="40" t="n"/>
+      <c r="H7" s="40" t="n"/>
+      <c r="I7" s="40" t="n"/>
+    </row>
+    <row r="8" ht="24" customHeight="1">
+      <c r="B8" s="41" t="inlineStr">
+        <is>
+          <t>Dampak Primer</t>
+        </is>
+      </c>
+      <c r="C8" s="42" t="n"/>
+      <c r="D8" s="42" t="n"/>
+      <c r="E8" s="42" t="n"/>
+      <c r="F8" s="42" t="n"/>
+      <c r="G8" s="42" t="n"/>
+      <c r="H8" s="42" t="n"/>
+      <c r="I8" s="43" t="n"/>
+    </row>
+    <row r="9" ht="36" customHeight="1">
+      <c r="B9" s="44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" s="44" t="inlineStr">
+        <is>
+          <t>GWP — Potensi pemanasan global</t>
+        </is>
+      </c>
+      <c r="D9" s="45" t="inlineStr">
+        <is>
+          <t>5. Overburden Removal
+Proses tidak dipadankan: dasar GWP HULU PROC dan LCI berbeda</t>
+        </is>
+      </c>
+      <c r="E9" s="46" t="inlineStr">
+        <is>
+          <t>Carbon dioxide, fossil
+[Air]</t>
+        </is>
+      </c>
+      <c r="F9" s="47" t="n">
+        <v>15.859743</v>
+      </c>
+      <c r="G9" s="46" t="inlineStr">
+        <is>
+          <t>kg CO2-eq</t>
+        </is>
+      </c>
+      <c r="H9" s="48" t="n">
+        <v>0.8564597226278381</v>
+      </c>
+      <c r="I9" s="48" t="n">
+        <v>0.8564597226278381</v>
+      </c>
+    </row>
+    <row r="10" ht="36" customHeight="1">
+      <c r="B10" s="44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" s="44" t="inlineStr">
+        <is>
+          <t>ODP — Potensi penipisan lapisan ozon</t>
+        </is>
+      </c>
+      <c r="D10" s="45" t="inlineStr">
+        <is>
+          <t>5. Overburden Removal
+Diesel {RoW}| diesel production, petroleum refinery operation | Cut-off, S</t>
+        </is>
+      </c>
+      <c r="E10" s="46" t="inlineStr">
+        <is>
+          <t>Methane, bromotrifluoro-, Halon 1301
+[Air]</t>
+        </is>
+      </c>
+      <c r="F10" s="47" t="n">
+        <v>1.8126076e-06</v>
+      </c>
+      <c r="G10" s="46" t="inlineStr">
+        <is>
+          <t>kg CFC-11 eq</t>
+        </is>
+      </c>
+      <c r="H10" s="48" t="n">
+        <v>0.9007719791218172</v>
+      </c>
+      <c r="I10" s="48" t="n">
+        <v>0.9007719791218172</v>
+      </c>
+    </row>
+    <row r="11" ht="36" customHeight="1">
+      <c r="B11" s="44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" s="44" t="inlineStr">
+        <is>
+          <t>AP — Potensi hujan asam</t>
+        </is>
+      </c>
+      <c r="D11" s="45" t="inlineStr">
+        <is>
+          <t>5. Overburden Removal
+5. Overburden Removal</t>
+        </is>
+      </c>
+      <c r="E11" s="46" t="inlineStr">
+        <is>
+          <t>Sulfur dioxide, ID
+[Air]</t>
+        </is>
+      </c>
+      <c r="F11" s="47" t="n">
+        <v>0.06807202800000001</v>
+      </c>
+      <c r="G11" s="46" t="inlineStr">
+        <is>
+          <t>kg SO2 eq</t>
+        </is>
+      </c>
+      <c r="H11" s="48" t="n">
+        <v>0.5385920782246281</v>
+      </c>
+      <c r="I11" s="48" t="n">
+        <v>0.5385920782246281</v>
+      </c>
+    </row>
+    <row r="12" ht="36" customHeight="1">
+      <c r="B12" s="44" t="n">
+        <v>2</v>
+      </c>
+      <c r="C12" s="44" t="inlineStr">
+        <is>
+          <t>AP — Potensi hujan asam</t>
+        </is>
+      </c>
+      <c r="D12" s="45" t="inlineStr">
+        <is>
+          <t>5. Overburden Removal
+5. Overburden Removal</t>
+        </is>
+      </c>
+      <c r="E12" s="46" t="inlineStr">
+        <is>
+          <t>Nitrogen oxides, ID
+[Air]</t>
+        </is>
+      </c>
+      <c r="F12" s="47" t="n">
+        <v>0.024285467</v>
+      </c>
+      <c r="G12" s="46" t="inlineStr">
+        <is>
+          <t>kg SO2 eq</t>
+        </is>
+      </c>
+      <c r="H12" s="48" t="n">
+        <v>0.1921488242158089</v>
+      </c>
+      <c r="I12" s="48" t="n">
+        <v>0.730740902440437</v>
+      </c>
+    </row>
+    <row r="13" ht="36" customHeight="1">
+      <c r="B13" s="44" t="n">
+        <v>3</v>
+      </c>
+      <c r="C13" s="44" t="inlineStr">
+        <is>
+          <t>AP — Potensi hujan asam</t>
+        </is>
+      </c>
+      <c r="D13" s="45" t="inlineStr">
+        <is>
+          <t>5. Overburden Removal
+5. Overburden Removal</t>
+        </is>
+      </c>
+      <c r="E13" s="46" t="inlineStr">
+        <is>
+          <t>Sulfur dioxide
+[Air]</t>
+        </is>
+      </c>
+      <c r="F13" s="47" t="n">
+        <v>0.012775671</v>
+      </c>
+      <c r="G13" s="46" t="inlineStr">
+        <is>
+          <t>kg SO2 eq</t>
+        </is>
+      </c>
+      <c r="H13" s="48" t="n">
+        <v>0.1010822711878675</v>
+      </c>
+      <c r="I13" s="48" t="n">
+        <v>0.8318231736283045</v>
+      </c>
+    </row>
+    <row r="14" ht="36" customHeight="1">
+      <c r="B14" s="44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" s="44" t="inlineStr">
+        <is>
+          <t>EP — Potensi eutrofikasi</t>
+        </is>
+      </c>
+      <c r="D14" s="45" t="inlineStr">
+        <is>
+          <t>5. Overburden Removal
+Palm oil, crude {MY}| palm oil mill operation | Cut-off, S</t>
+        </is>
+      </c>
+      <c r="E14" s="46" t="inlineStr">
+        <is>
+          <t>Nitrate
+[Water]</t>
+        </is>
+      </c>
+      <c r="F14" s="47" t="n">
+        <v>0.015281975</v>
+      </c>
+      <c r="G14" s="46" t="inlineStr">
+        <is>
+          <t>kg PO4--- eq</t>
+        </is>
+      </c>
+      <c r="H14" s="48" t="n">
+        <v>0.5218902978105844</v>
+      </c>
+      <c r="I14" s="48" t="n">
+        <v>0.5218902978105844</v>
+      </c>
+    </row>
+    <row r="15" ht="36" customHeight="1">
+      <c r="B15" s="44" t="n">
+        <v>2</v>
+      </c>
+      <c r="C15" s="44" t="inlineStr">
+        <is>
+          <t>EP — Potensi eutrofikasi</t>
+        </is>
+      </c>
+      <c r="D15" s="45" t="inlineStr">
+        <is>
+          <t>5. Overburden Removal
+Palm oil, crude {MY}| palm oil mill operation | Cut-off, S</t>
+        </is>
+      </c>
+      <c r="E15" s="46" t="inlineStr">
+        <is>
+          <t>Nitrogen oxides, ID
+[Air]</t>
+        </is>
+      </c>
+      <c r="F15" s="47" t="n">
+        <v>0.0063142214</v>
+      </c>
+      <c r="G15" s="46" t="inlineStr">
+        <is>
+          <t>kg PO4--- eq</t>
+        </is>
+      </c>
+      <c r="H15" s="48" t="n">
+        <v>0.2156351444684319</v>
+      </c>
+      <c r="I15" s="48" t="n">
+        <v>0.7375254422790163</v>
+      </c>
+    </row>
+    <row r="16" ht="36" customHeight="1">
+      <c r="B16" s="44" t="n">
+        <v>3</v>
+      </c>
+      <c r="C16" s="44" t="inlineStr">
+        <is>
+          <t>EP — Potensi eutrofikasi</t>
+        </is>
+      </c>
+      <c r="D16" s="45" t="inlineStr">
+        <is>
+          <t>5. Overburden Removal
+Palm oil, crude {MY}| palm oil mill operation | Cut-off, S</t>
+        </is>
+      </c>
+      <c r="E16" s="46" t="inlineStr">
+        <is>
+          <t>Ammonia
+[Air]</t>
+        </is>
+      </c>
+      <c r="F16" s="47" t="n">
+        <v>0.0015604377</v>
+      </c>
+      <c r="G16" s="46" t="inlineStr">
+        <is>
+          <t>kg PO4--- eq</t>
+        </is>
+      </c>
+      <c r="H16" s="48" t="n">
+        <v>0.0532900555044661</v>
+      </c>
+      <c r="I16" s="48" t="n">
+        <v>0.7908154977834824</v>
+      </c>
+    </row>
+    <row r="17" ht="36" customHeight="1">
+      <c r="B17" s="44" t="n">
+        <v>4</v>
+      </c>
+      <c r="C17" s="44" t="inlineStr">
+        <is>
+          <t>EP — Potensi eutrofikasi</t>
+        </is>
+      </c>
+      <c r="D17" s="45" t="inlineStr">
+        <is>
+          <t>5. Overburden Removal
+Palm oil, crude {MY}| palm oil mill operation | Cut-off, S</t>
+        </is>
+      </c>
+      <c r="E17" s="46" t="inlineStr">
+        <is>
+          <t>Nitrogen oxides
+[Air]</t>
+        </is>
+      </c>
+      <c r="F17" s="47" t="n">
+        <v>0.0011870125</v>
+      </c>
+      <c r="G17" s="46" t="inlineStr">
+        <is>
+          <t>kg PO4--- eq</t>
+        </is>
+      </c>
+      <c r="H17" s="48" t="n">
+        <v>0.0405373197593823</v>
+      </c>
+      <c r="I17" s="48" t="n">
+        <v>0.8313528175428646</v>
+      </c>
+    </row>
+    <row r="18" ht="24" customHeight="1">
+      <c r="B18" s="41" t="inlineStr">
+        <is>
+          <t>Dampak Sekunder</t>
+        </is>
+      </c>
+      <c r="C18" s="42" t="n"/>
+      <c r="D18" s="42" t="n"/>
+      <c r="E18" s="42" t="n"/>
+      <c r="F18" s="42" t="n"/>
+      <c r="G18" s="42" t="n"/>
+      <c r="H18" s="42" t="n"/>
+      <c r="I18" s="43" t="n"/>
+    </row>
+    <row r="19" ht="36" customHeight="1">
+      <c r="B19" s="44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C19" s="44" t="inlineStr">
+        <is>
+          <t>POFP — Photochemical oxidation</t>
+        </is>
+      </c>
+      <c r="D19" s="45" t="inlineStr">
+        <is>
+          <t>5. Overburden Removal
+5. Overburden Removal</t>
+        </is>
+      </c>
+      <c r="E19" s="46" t="inlineStr">
+        <is>
+          <t>Carbon monoxide, fossil
+[Air]</t>
+        </is>
+      </c>
+      <c r="F19" s="47" t="n">
+        <v>0.0042368308</v>
+      </c>
+      <c r="G19" s="46" t="inlineStr">
+        <is>
+          <t>kg C2H4 eq</t>
+        </is>
+      </c>
+      <c r="H19" s="48" t="n">
+        <v>0.3733502735558667</v>
+      </c>
+      <c r="I19" s="48" t="n">
+        <v>0.3733502735558667</v>
+      </c>
+    </row>
+    <row r="20" ht="36" customHeight="1">
+      <c r="B20" s="44" t="n">
+        <v>2</v>
+      </c>
+      <c r="C20" s="44" t="inlineStr">
+        <is>
+          <t>POFP — Photochemical oxidation</t>
+        </is>
+      </c>
+      <c r="D20" s="45" t="inlineStr">
+        <is>
+          <t>5. Overburden Removal
+5. Overburden Removal</t>
+        </is>
+      </c>
+      <c r="E20" s="46" t="inlineStr">
+        <is>
+          <t>Sulfur dioxide, ID
+[Air]</t>
+        </is>
+      </c>
+      <c r="F20" s="47" t="n">
+        <v>0.0027228811</v>
+      </c>
+      <c r="G20" s="46" t="inlineStr">
+        <is>
+          <t>kg C2H4 eq</t>
+        </is>
+      </c>
+      <c r="H20" s="48" t="n">
+        <v>0.2399407603308349</v>
+      </c>
+      <c r="I20" s="48" t="n">
+        <v>0.6132910338867016</v>
+      </c>
+    </row>
+    <row r="21" ht="36" customHeight="1">
+      <c r="B21" s="44" t="n">
+        <v>3</v>
+      </c>
+      <c r="C21" s="44" t="inlineStr">
+        <is>
+          <t>POFP — Photochemical oxidation</t>
+        </is>
+      </c>
+      <c r="D21" s="45" t="inlineStr">
+        <is>
+          <t>5. Overburden Removal
+5. Overburden Removal</t>
+        </is>
+      </c>
+      <c r="E21" s="46" t="inlineStr">
+        <is>
+          <t>Hexane
+[Air]</t>
+        </is>
+      </c>
+      <c r="F21" s="47" t="n">
+        <v>0.0021400412</v>
+      </c>
+      <c r="G21" s="46" t="inlineStr">
+        <is>
+          <t>kg C2H4 eq</t>
+        </is>
+      </c>
+      <c r="H21" s="48" t="n">
+        <v>0.1885808060687308</v>
+      </c>
+      <c r="I21" s="48" t="n">
+        <v>0.8018718399554323</v>
+      </c>
+    </row>
+    <row r="22" ht="36" customHeight="1">
+      <c r="B22" s="44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C22" s="44" t="inlineStr">
+        <is>
+          <t>ABF — Abiotic depletion (fossil fuels)</t>
+        </is>
+      </c>
+      <c r="D22" s="45" t="inlineStr">
+        <is>
+          <t>5. Overburden Removal
+Diesel {RoW}| diesel production, petroleum refinery operation | Cut-off, S</t>
+        </is>
+      </c>
+      <c r="E22" s="46" t="inlineStr">
+        <is>
+          <t>Oil, crude
+[Raw]</t>
+        </is>
+      </c>
+      <c r="F22" s="47" t="n">
+        <v>131.21262</v>
+      </c>
+      <c r="G22" s="46" t="inlineStr">
+        <is>
+          <t>MJ</t>
+        </is>
+      </c>
+      <c r="H22" s="48" t="n">
+        <v>0.7839608669080181</v>
+      </c>
+      <c r="I22" s="48" t="n">
+        <v>0.7839608669080181</v>
+      </c>
+    </row>
+    <row r="23" ht="36" customHeight="1">
+      <c r="B23" s="44" t="n">
+        <v>2</v>
+      </c>
+      <c r="C23" s="44" t="inlineStr">
+        <is>
+          <t>ABF — Abiotic depletion (fossil fuels)</t>
+        </is>
+      </c>
+      <c r="D23" s="45" t="inlineStr">
+        <is>
+          <t>5. Overburden Removal
+Diesel {RoW}| diesel production, petroleum refinery operation | Cut-off, S</t>
+        </is>
+      </c>
+      <c r="E23" s="46" t="inlineStr">
+        <is>
+          <t>Gas, natural/m3
+[Raw]</t>
+        </is>
+      </c>
+      <c r="F23" s="47" t="n">
+        <v>10.833072</v>
+      </c>
+      <c r="G23" s="46" t="inlineStr">
+        <is>
+          <t>MJ</t>
+        </is>
+      </c>
+      <c r="H23" s="48" t="n">
+        <v>0.06472475373479303</v>
+      </c>
+      <c r="I23" s="48" t="n">
+        <v>0.8486856206428112</v>
+      </c>
+    </row>
+    <row r="24" ht="36" customHeight="1">
+      <c r="B24" s="44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C24" s="44" t="inlineStr">
+        <is>
+          <t>ABN — Abiotic depletion</t>
+        </is>
+      </c>
+      <c r="D24" s="45" t="inlineStr">
+        <is>
+          <t>1. Supporting Material Production and Transportation
+Ammonium nitrate {RoW}| market for ammonium nitrate | Cut-off, S</t>
+        </is>
+      </c>
+      <c r="E24" s="46" t="inlineStr">
+        <is>
+          <t>Tellurium
+[Raw]</t>
+        </is>
+      </c>
+      <c r="F24" s="47" t="n">
+        <v>1.1484751e-05</v>
+      </c>
+      <c r="G24" s="46" t="inlineStr">
+        <is>
+          <t>kg Sb eq</t>
+        </is>
+      </c>
+      <c r="H24" s="48" t="n">
+        <v>0.3062930164664935</v>
+      </c>
+      <c r="I24" s="48" t="n">
+        <v>0.3062930164664935</v>
+      </c>
+    </row>
+    <row r="25" ht="36" customHeight="1">
+      <c r="B25" s="44" t="n">
+        <v>2</v>
+      </c>
+      <c r="C25" s="44" t="inlineStr">
+        <is>
+          <t>ABN — Abiotic depletion</t>
+        </is>
+      </c>
+      <c r="D25" s="45" t="inlineStr">
+        <is>
+          <t>5. Overburden Removal
+Palm oil, crude {MY}| palm oil mill operation | Cut-off, S</t>
+        </is>
+      </c>
+      <c r="E25" s="46" t="inlineStr">
+        <is>
+          <t>Tellurium
+[Raw]</t>
+        </is>
+      </c>
+      <c r="F25" s="47" t="n">
+        <v>6.2221474e-06</v>
+      </c>
+      <c r="G25" s="46" t="inlineStr">
+        <is>
+          <t>kg Sb eq</t>
+        </is>
+      </c>
+      <c r="H25" s="48" t="n">
+        <v>0.1659418037052044</v>
+      </c>
+      <c r="I25" s="48" t="n">
+        <v>0.4722348201716979</v>
+      </c>
+    </row>
+    <row r="26" ht="36" customHeight="1">
+      <c r="B26" s="44" t="n">
+        <v>3</v>
+      </c>
+      <c r="C26" s="44" t="inlineStr">
+        <is>
+          <t>ABN — Abiotic depletion</t>
+        </is>
+      </c>
+      <c r="D26" s="45" t="inlineStr">
+        <is>
+          <t>5. Overburden Removal
+Palm oil, crude {MY}| palm oil mill operation | Cut-off, S</t>
+        </is>
+      </c>
+      <c r="E26" s="46" t="inlineStr">
+        <is>
+          <t>Lead
+[Raw]</t>
+        </is>
+      </c>
+      <c r="F26" s="47" t="n">
+        <v>4.0121112e-06</v>
+      </c>
+      <c r="G26" s="46" t="inlineStr">
+        <is>
+          <t>kg Sb eq</t>
+        </is>
+      </c>
+      <c r="H26" s="48" t="n">
+        <v>0.1070011567379217</v>
+      </c>
+      <c r="I26" s="48" t="n">
+        <v>0.5792359769096196</v>
+      </c>
+    </row>
+    <row r="27" ht="36" customHeight="1">
+      <c r="B27" s="44" t="n">
+        <v>4</v>
+      </c>
+      <c r="C27" s="44" t="inlineStr">
+        <is>
+          <t>ABN — Abiotic depletion</t>
+        </is>
+      </c>
+      <c r="D27" s="45" t="inlineStr">
+        <is>
+          <t>1. Supporting Material Production and Transportation
+Ammonium nitrate {RoW}| market for ammonium nitrate | Cut-off, S</t>
+        </is>
+      </c>
+      <c r="E27" s="46" t="inlineStr">
+        <is>
+          <t>Gold
+[Raw]</t>
+        </is>
+      </c>
+      <c r="F27" s="47" t="n">
+        <v>2.9034454e-06</v>
+      </c>
+      <c r="G27" s="46" t="inlineStr">
+        <is>
+          <t>kg Sb eq</t>
+        </is>
+      </c>
+      <c r="H27" s="48" t="n">
+        <v>0.07743355077630894</v>
+      </c>
+      <c r="I27" s="48" t="n">
+        <v>0.6566695276859286</v>
+      </c>
+    </row>
+    <row r="28" ht="36" customHeight="1">
+      <c r="B28" s="44" t="n">
+        <v>5</v>
+      </c>
+      <c r="C28" s="44" t="inlineStr">
+        <is>
+          <t>ABN — Abiotic depletion</t>
+        </is>
+      </c>
+      <c r="D28" s="45" t="inlineStr">
+        <is>
+          <t>5. Overburden Removal
+Palm oil, crude {MY}| palm oil mill operation | Cut-off, S</t>
+        </is>
+      </c>
+      <c r="E28" s="46" t="inlineStr">
+        <is>
+          <t>Silver
+[Raw]</t>
+        </is>
+      </c>
+      <c r="F28" s="47" t="n">
+        <v>2.0370715e-06</v>
+      </c>
+      <c r="G28" s="46" t="inlineStr">
+        <is>
+          <t>kg Sb eq</t>
+        </is>
+      </c>
+      <c r="H28" s="48" t="n">
+        <v>0.05432775812840215</v>
+      </c>
+      <c r="I28" s="48" t="n">
+        <v>0.7109972858143307</v>
+      </c>
+    </row>
+    <row r="29" ht="36" customHeight="1">
+      <c r="B29" s="44" t="n">
+        <v>6</v>
+      </c>
+      <c r="C29" s="44" t="inlineStr">
+        <is>
+          <t>ABN — Abiotic depletion</t>
+        </is>
+      </c>
+      <c r="D29" s="45" t="inlineStr">
+        <is>
+          <t>1. Supporting Material Production and Transportation
+Ammonium nitrate {RoW}| market for ammonium nitrate | Cut-off, S</t>
+        </is>
+      </c>
+      <c r="E29" s="46" t="inlineStr">
+        <is>
+          <t>Silver
+[Raw]</t>
+        </is>
+      </c>
+      <c r="F29" s="47" t="n">
+        <v>1.6951678e-06</v>
+      </c>
+      <c r="G29" s="46" t="inlineStr">
+        <is>
+          <t>kg Sb eq</t>
+        </is>
+      </c>
+      <c r="H29" s="48" t="n">
+        <v>0.04520934401441264</v>
+      </c>
+      <c r="I29" s="48" t="n">
+        <v>0.7562066298287434</v>
+      </c>
+    </row>
+    <row r="30" ht="36" customHeight="1">
+      <c r="B30" s="44" t="n">
+        <v>7</v>
+      </c>
+      <c r="C30" s="44" t="inlineStr">
+        <is>
+          <t>ABN — Abiotic depletion</t>
+        </is>
+      </c>
+      <c r="D30" s="45" t="inlineStr">
+        <is>
+          <t>5. Overburden Removal
+Palm oil, crude {MY}| palm oil mill operation | Cut-off, S</t>
+        </is>
+      </c>
+      <c r="E30" s="46" t="inlineStr">
+        <is>
+          <t>Zinc
+[Raw]</t>
+        </is>
+      </c>
+      <c r="F30" s="47" t="n">
+        <v>1.5778647e-06</v>
+      </c>
+      <c r="G30" s="46" t="inlineStr">
+        <is>
+          <t>kg Sb eq</t>
+        </is>
+      </c>
+      <c r="H30" s="48" t="n">
+        <v>0.04208092439609695</v>
+      </c>
+      <c r="I30" s="48" t="n">
+        <v>0.7982875542248404</v>
+      </c>
+    </row>
+    <row r="31" ht="36" customHeight="1">
+      <c r="B31" s="44" t="n">
+        <v>8</v>
+      </c>
+      <c r="C31" s="44" t="inlineStr">
+        <is>
+          <t>ABN — Abiotic depletion</t>
+        </is>
+      </c>
+      <c r="D31" s="45" t="inlineStr">
+        <is>
+          <t>1. Supporting Material Production and Transportation
+Ammonium nitrate {RoW}| market for ammonium nitrate | Cut-off, S</t>
+        </is>
+      </c>
+      <c r="E31" s="46" t="inlineStr">
+        <is>
+          <t>Copper
+[Raw]</t>
+        </is>
+      </c>
+      <c r="F31" s="47" t="n">
+        <v>1.2794853e-06</v>
+      </c>
+      <c r="G31" s="46" t="inlineStr">
+        <is>
+          <t>kg Sb eq</t>
+        </is>
+      </c>
+      <c r="H31" s="48" t="n">
+        <v>0.03412328330510051</v>
+      </c>
+      <c r="I31" s="48" t="n">
+        <v>0.8324108375299409</v>
+      </c>
+    </row>
+    <row r="32" ht="36" customHeight="1">
+      <c r="B32" s="44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C32" s="44" t="inlineStr">
+        <is>
+          <t>ETP Terrestrial — Ecotoxicity — Terrestrial</t>
+        </is>
+      </c>
+      <c r="D32" s="45" t="inlineStr">
+        <is>
+          <t>5. Overburden Removal
+Palm oil, crude {MY}| palm oil mill operation | Cut-off, S</t>
+        </is>
+      </c>
+      <c r="E32" s="46" t="inlineStr">
+        <is>
+          <t>Copper
+[Air]</t>
+        </is>
+      </c>
+      <c r="F32" s="47" t="n">
+        <v>4.0438757</v>
+      </c>
+      <c r="G32" s="46" t="inlineStr">
+        <is>
+          <t>kg 1,4-DCB</t>
+        </is>
+      </c>
+      <c r="H32" s="48" t="n">
+        <v>0.2699302778832063</v>
+      </c>
+      <c r="I32" s="48" t="n">
+        <v>0.2699302778832063</v>
+      </c>
+    </row>
+    <row r="33" ht="36" customHeight="1">
+      <c r="B33" s="44" t="n">
+        <v>2</v>
+      </c>
+      <c r="C33" s="44" t="inlineStr">
+        <is>
+          <t>ETP Terrestrial — Ecotoxicity — Terrestrial</t>
+        </is>
+      </c>
+      <c r="D33" s="45" t="inlineStr">
+        <is>
+          <t>1. Supporting Material Production and Transportation
+Ammonium nitrate {RoW}| market for ammonium nitrate | Cut-off, S</t>
+        </is>
+      </c>
+      <c r="E33" s="46" t="inlineStr">
+        <is>
+          <t>Copper
+[Air]</t>
+        </is>
+      </c>
+      <c r="F33" s="47" t="n">
+        <v>3.7129873</v>
+      </c>
+      <c r="G33" s="46" t="inlineStr">
+        <is>
+          <t>kg 1,4-DCB</t>
+        </is>
+      </c>
+      <c r="H33" s="48" t="n">
+        <v>0.2478433483170158</v>
+      </c>
+      <c r="I33" s="48" t="n">
+        <v>0.5177736262002222</v>
+      </c>
+    </row>
+    <row r="34" ht="36" customHeight="1">
+      <c r="B34" s="44" t="n">
+        <v>3</v>
+      </c>
+      <c r="C34" s="44" t="inlineStr">
+        <is>
+          <t>ETP Terrestrial — Ecotoxicity — Terrestrial</t>
+        </is>
+      </c>
+      <c r="D34" s="45" t="inlineStr">
+        <is>
+          <t>5. Overburden Removal
+Palm oil, crude {MY}| palm oil mill operation | Cut-off, S</t>
+        </is>
+      </c>
+      <c r="E34" s="46" t="inlineStr">
+        <is>
+          <t>Vanadium
+[Air]</t>
+        </is>
+      </c>
+      <c r="F34" s="47" t="n">
+        <v>1.9929989</v>
+      </c>
+      <c r="G34" s="46" t="inlineStr">
+        <is>
+          <t>kg 1,4-DCB</t>
+        </is>
+      </c>
+      <c r="H34" s="48" t="n">
+        <v>0.1330334527586801</v>
+      </c>
+      <c r="I34" s="48" t="n">
+        <v>0.6508070789589022</v>
+      </c>
+    </row>
+    <row r="35" ht="36" customHeight="1">
+      <c r="B35" s="44" t="n">
+        <v>4</v>
+      </c>
+      <c r="C35" s="44" t="inlineStr">
+        <is>
+          <t>ETP Terrestrial — Ecotoxicity — Terrestrial</t>
+        </is>
+      </c>
+      <c r="D35" s="45" t="inlineStr">
+        <is>
+          <t>5. Overburden Removal
+Palm oil, crude {MY}| palm oil mill operation | Cut-off, S</t>
+        </is>
+      </c>
+      <c r="E35" s="46" t="inlineStr">
+        <is>
+          <t>Zinc
+[Air]</t>
+        </is>
+      </c>
+      <c r="F35" s="47" t="n">
+        <v>1.3026289</v>
+      </c>
+      <c r="G35" s="46" t="inlineStr">
+        <is>
+          <t>kg 1,4-DCB</t>
+        </is>
+      </c>
+      <c r="H35" s="48" t="n">
+        <v>0.0869509863905301</v>
+      </c>
+      <c r="I35" s="48" t="n">
+        <v>0.7377580653494323</v>
+      </c>
+    </row>
+    <row r="36" ht="36" customHeight="1">
+      <c r="B36" s="44" t="n">
+        <v>5</v>
+      </c>
+      <c r="C36" s="44" t="inlineStr">
+        <is>
+          <t>ETP Terrestrial — Ecotoxicity — Terrestrial</t>
+        </is>
+      </c>
+      <c r="D36" s="45" t="inlineStr">
+        <is>
+          <t>5. Overburden Removal
+Palm oil, crude {MY}| palm oil mill operation | Cut-off, S</t>
+        </is>
+      </c>
+      <c r="E36" s="46" t="inlineStr">
+        <is>
+          <t>Nickel
+[Air]</t>
+        </is>
+      </c>
+      <c r="F36" s="47" t="n">
+        <v>1.2656046</v>
+      </c>
+      <c r="G36" s="46" t="inlineStr">
+        <is>
+          <t>kg 1,4-DCB</t>
+        </is>
+      </c>
+      <c r="H36" s="48" t="n">
+        <v>0.08447959994622589</v>
+      </c>
+      <c r="I36" s="48" t="n">
+        <v>0.8222376652956582</v>
+      </c>
+    </row>
+    <row r="37" ht="36" customHeight="1">
+      <c r="B37" s="44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C37" s="44" t="inlineStr">
+        <is>
+          <t>ETP Freshwater — Ecotoxicity — Freshwater</t>
+        </is>
+      </c>
+      <c r="D37" s="45" t="inlineStr">
+        <is>
+          <t>5. Overburden Removal
+Palm oil, crude {MY}| palm oil mill operation | Cut-off, S</t>
+        </is>
+      </c>
+      <c r="E37" s="46" t="inlineStr">
+        <is>
+          <t>Carbofuran
+[Soil]</t>
+        </is>
+      </c>
+      <c r="F37" s="47" t="n">
+        <v>0.0054697634</v>
+      </c>
+      <c r="G37" s="46" t="inlineStr">
+        <is>
+          <t>kg 1,4-DCB</t>
+        </is>
+      </c>
+      <c r="H37" s="48" t="n">
+        <v>0.3088649253799189</v>
+      </c>
+      <c r="I37" s="48" t="n">
+        <v>0.3088649253799189</v>
+      </c>
+    </row>
+    <row r="38" ht="36" customHeight="1">
+      <c r="B38" s="44" t="n">
+        <v>2</v>
+      </c>
+      <c r="C38" s="44" t="inlineStr">
+        <is>
+          <t>ETP Freshwater — Ecotoxicity — Freshwater</t>
+        </is>
+      </c>
+      <c r="D38" s="45" t="inlineStr">
+        <is>
+          <t>5. Overburden Removal
+Palm oil, crude {MY}| palm oil mill operation | Cut-off, S</t>
+        </is>
+      </c>
+      <c r="E38" s="46" t="inlineStr">
+        <is>
+          <t>Zinc
+[Water]</t>
+        </is>
+      </c>
+      <c r="F38" s="47" t="n">
+        <v>0.0029894239</v>
+      </c>
+      <c r="G38" s="46" t="inlineStr">
+        <is>
+          <t>kg 1,4-DCB</t>
+        </is>
+      </c>
+      <c r="H38" s="48" t="n">
+        <v>0.1688058737243454</v>
+      </c>
+      <c r="I38" s="48" t="n">
+        <v>0.4776707991042642</v>
+      </c>
+    </row>
+    <row r="39" ht="36" customHeight="1">
+      <c r="B39" s="44" t="n">
+        <v>3</v>
+      </c>
+      <c r="C39" s="44" t="inlineStr">
+        <is>
+          <t>ETP Freshwater — Ecotoxicity — Freshwater</t>
+        </is>
+      </c>
+      <c r="D39" s="45" t="inlineStr">
+        <is>
+          <t>5. Overburden Removal
+Palm oil, crude {MY}| palm oil mill operation | Cut-off, S</t>
+        </is>
+      </c>
+      <c r="E39" s="46" t="inlineStr">
+        <is>
+          <t>Cypermethrin
+[Soil]</t>
+        </is>
+      </c>
+      <c r="F39" s="47" t="n">
+        <v>0.0021255276</v>
+      </c>
+      <c r="G39" s="46" t="inlineStr">
+        <is>
+          <t>kg 1,4-DCB</t>
+        </is>
+      </c>
+      <c r="H39" s="48" t="n">
+        <v>0.1200236418940823</v>
+      </c>
+      <c r="I39" s="48" t="n">
+        <v>0.5976944409983466</v>
+      </c>
+    </row>
+    <row r="40" ht="36" customHeight="1">
+      <c r="B40" s="44" t="n">
+        <v>4</v>
+      </c>
+      <c r="C40" s="44" t="inlineStr">
+        <is>
+          <t>ETP Freshwater — Ecotoxicity — Freshwater</t>
+        </is>
+      </c>
+      <c r="D40" s="45" t="inlineStr">
+        <is>
+          <t>1. Supporting Material Production and Transportation
+Textile, knit cotton {GLO}| market for | Cut-off, S</t>
+        </is>
+      </c>
+      <c r="E40" s="46" t="inlineStr">
+        <is>
+          <t>Chlorpyrifos
+[Soil]</t>
+        </is>
+      </c>
+      <c r="F40" s="47" t="n">
+        <v>0.001563263</v>
+      </c>
+      <c r="G40" s="46" t="inlineStr">
+        <is>
+          <t>kg 1,4-DCB</t>
+        </is>
+      </c>
+      <c r="H40" s="48" t="n">
+        <v>0.08827385657013759</v>
+      </c>
+      <c r="I40" s="48" t="n">
+        <v>0.6859682975684842</v>
+      </c>
+    </row>
+    <row r="41" ht="36" customHeight="1">
+      <c r="B41" s="44" t="n">
+        <v>5</v>
+      </c>
+      <c r="C41" s="44" t="inlineStr">
+        <is>
+          <t>ETP Freshwater — Ecotoxicity — Freshwater</t>
+        </is>
+      </c>
+      <c r="D41" s="45" t="inlineStr">
+        <is>
+          <t>1. Supporting Material Production and Transportation
+Textile, knit cotton {GLO}| market for | Cut-off, S</t>
+        </is>
+      </c>
+      <c r="E41" s="46" t="inlineStr">
+        <is>
+          <t>Profenofos
+[Soil]</t>
+        </is>
+      </c>
+      <c r="F41" s="47" t="n">
+        <v>0.0014086182</v>
+      </c>
+      <c r="G41" s="46" t="inlineStr">
+        <is>
+          <t>kg 1,4-DCB</t>
+        </is>
+      </c>
+      <c r="H41" s="48" t="n">
+        <v>0.0795414213404177</v>
+      </c>
+      <c r="I41" s="48" t="n">
+        <v>0.765509718908902</v>
+      </c>
+    </row>
+    <row r="42" ht="36" customHeight="1">
+      <c r="B42" s="44" t="n">
+        <v>6</v>
+      </c>
+      <c r="C42" s="44" t="inlineStr">
+        <is>
+          <t>ETP Freshwater — Ecotoxicity — Freshwater</t>
+        </is>
+      </c>
+      <c r="D42" s="45" t="inlineStr">
+        <is>
+          <t>1. Supporting Material Production and Transportation
+Textile, knit cotton {GLO}| market for | Cut-off, S</t>
+        </is>
+      </c>
+      <c r="E42" s="46" t="inlineStr">
+        <is>
+          <t>Zinc
+[Water]</t>
+        </is>
+      </c>
+      <c r="F42" s="47" t="n">
+        <v>0.00071192332</v>
+      </c>
+      <c r="G42" s="46" t="inlineStr">
+        <is>
+          <t>kg 1,4-DCB</t>
+        </is>
+      </c>
+      <c r="H42" s="48" t="n">
+        <v>0.04020066811446069</v>
+      </c>
+      <c r="I42" s="48" t="n">
+        <v>0.8057103870233626</v>
+      </c>
+    </row>
+    <row r="43" ht="36" customHeight="1">
+      <c r="B43" s="44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C43" s="44" t="inlineStr">
+        <is>
+          <t>ETP Marine — Ecotoxicity — Marine</t>
+        </is>
+      </c>
+      <c r="D43" s="45" t="inlineStr">
+        <is>
+          <t>5. Overburden Removal
+Diesel {RoW}| diesel production, petroleum refinery operation | Cut-off, S</t>
+        </is>
+      </c>
+      <c r="E43" s="46" t="inlineStr">
+        <is>
+          <t>Zinc
+[Water]</t>
+        </is>
+      </c>
+      <c r="F43" s="47" t="n">
+        <v>0.008038019699999999</v>
+      </c>
+      <c r="G43" s="46" t="inlineStr">
+        <is>
+          <t>kg 1,4-DCB</t>
+        </is>
+      </c>
+      <c r="H43" s="48" t="n">
+        <v>0.3371484125939849</v>
+      </c>
+      <c r="I43" s="48" t="n">
+        <v>0.3371484125939849</v>
+      </c>
+    </row>
+    <row r="44" ht="36" customHeight="1">
+      <c r="B44" s="44" t="n">
+        <v>2</v>
+      </c>
+      <c r="C44" s="44" t="inlineStr">
+        <is>
+          <t>ETP Marine — Ecotoxicity — Marine</t>
+        </is>
+      </c>
+      <c r="D44" s="45" t="inlineStr">
+        <is>
+          <t>5. Overburden Removal
+Diesel {RoW}| diesel production, petroleum refinery operation | Cut-off, S</t>
+        </is>
+      </c>
+      <c r="E44" s="46" t="inlineStr">
+        <is>
+          <t>Copper
+[Air]</t>
+        </is>
+      </c>
+      <c r="F44" s="47" t="n">
+        <v>0.0016952175</v>
+      </c>
+      <c r="G44" s="46" t="inlineStr">
+        <is>
+          <t>kg 1,4-DCB</t>
+        </is>
+      </c>
+      <c r="H44" s="48" t="n">
+        <v>0.07110456436509401</v>
+      </c>
+      <c r="I44" s="48" t="n">
+        <v>0.4082529769590789</v>
+      </c>
+    </row>
+    <row r="45" ht="36" customHeight="1">
+      <c r="B45" s="44" t="n">
+        <v>3</v>
+      </c>
+      <c r="C45" s="44" t="inlineStr">
+        <is>
+          <t>ETP Marine — Ecotoxicity — Marine</t>
+        </is>
+      </c>
+      <c r="D45" s="45" t="inlineStr">
+        <is>
+          <t>5. Overburden Removal
+Diesel {RoW}| diesel production, petroleum refinery operation | Cut-off, S</t>
+        </is>
+      </c>
+      <c r="E45" s="46" t="inlineStr">
+        <is>
+          <t>Cypermethrin
+[Soil]</t>
+        </is>
+      </c>
+      <c r="F45" s="47" t="n">
+        <v>0.001683342</v>
+      </c>
+      <c r="G45" s="46" t="inlineStr">
+        <is>
+          <t>kg 1,4-DCB</t>
+        </is>
+      </c>
+      <c r="H45" s="48" t="n">
+        <v>0.07060645586036368</v>
+      </c>
+      <c r="I45" s="48" t="n">
+        <v>0.4788594328194425</v>
+      </c>
+    </row>
+    <row r="46" ht="36" customHeight="1">
+      <c r="B46" s="44" t="n">
+        <v>4</v>
+      </c>
+      <c r="C46" s="44" t="inlineStr">
+        <is>
+          <t>ETP Marine — Ecotoxicity — Marine</t>
+        </is>
+      </c>
+      <c r="D46" s="45" t="inlineStr">
+        <is>
+          <t>5. Overburden Removal
+Diesel {RoW}| diesel production, petroleum refinery operation | Cut-off, S</t>
+        </is>
+      </c>
+      <c r="E46" s="46" t="inlineStr">
+        <is>
+          <t>Vanadium
+[Air]</t>
+        </is>
+      </c>
+      <c r="F46" s="47" t="n">
+        <v>0.0016410983</v>
+      </c>
+      <c r="G46" s="46" t="inlineStr">
+        <is>
+          <t>kg 1,4-DCB</t>
+        </is>
+      </c>
+      <c r="H46" s="48" t="n">
+        <v>0.06883457709809883</v>
+      </c>
+      <c r="I46" s="48" t="n">
+        <v>0.5476940099175414</v>
+      </c>
+    </row>
+    <row r="47" ht="36" customHeight="1">
+      <c r="B47" s="44" t="n">
+        <v>5</v>
+      </c>
+      <c r="C47" s="44" t="inlineStr">
+        <is>
+          <t>ETP Marine — Ecotoxicity — Marine</t>
+        </is>
+      </c>
+      <c r="D47" s="45" t="inlineStr">
+        <is>
+          <t>1. Supporting Material Production and Transportation
+Ammonium nitrate {RoW}| market for ammonium nitrate | Cut-off, S</t>
+        </is>
+      </c>
+      <c r="E47" s="46" t="inlineStr">
+        <is>
+          <t>Copper
+[Air]</t>
+        </is>
+      </c>
+      <c r="F47" s="47" t="n">
+        <v>0.0015543174</v>
+      </c>
+      <c r="G47" s="46" t="inlineStr">
+        <is>
+          <t>kg 1,4-DCB</t>
+        </is>
+      </c>
+      <c r="H47" s="48" t="n">
+        <v>0.06519462052042618</v>
+      </c>
+      <c r="I47" s="48" t="n">
+        <v>0.6128886304379675</v>
+      </c>
+    </row>
+    <row r="48" ht="36" customHeight="1">
+      <c r="B48" s="44" t="n">
+        <v>6</v>
+      </c>
+      <c r="C48" s="44" t="inlineStr">
+        <is>
+          <t>ETP Marine — Ecotoxicity — Marine</t>
+        </is>
+      </c>
+      <c r="D48" s="45" t="inlineStr">
+        <is>
+          <t>1. Supporting Material Production and Transportation
+Ammonium nitrate {RoW}| market for ammonium nitrate | Cut-off, S</t>
+        </is>
+      </c>
+      <c r="E48" s="46" t="inlineStr">
+        <is>
+          <t>Zinc
+[Water]</t>
+        </is>
+      </c>
+      <c r="F48" s="47" t="n">
+        <v>0.0015323501</v>
+      </c>
+      <c r="G48" s="46" t="inlineStr">
+        <is>
+          <t>kg 1,4-DCB</t>
+        </is>
+      </c>
+      <c r="H48" s="48" t="n">
+        <v>0.06427321940418161</v>
+      </c>
+      <c r="I48" s="48" t="n">
+        <v>0.6771618498421491</v>
+      </c>
+    </row>
+    <row r="49" ht="36" customHeight="1">
+      <c r="B49" s="44" t="n">
+        <v>7</v>
+      </c>
+      <c r="C49" s="44" t="inlineStr">
+        <is>
+          <t>ETP Marine — Ecotoxicity — Marine</t>
+        </is>
+      </c>
+      <c r="D49" s="45" t="inlineStr">
+        <is>
+          <t>5. Overburden Removal
+Diesel {RoW}| diesel production, petroleum refinery operation | Cut-off, S</t>
+        </is>
+      </c>
+      <c r="E49" s="46" t="inlineStr">
+        <is>
+          <t>Zinc
+[Air]</t>
+        </is>
+      </c>
+      <c r="F49" s="47" t="n">
+        <v>0.0011104678</v>
+      </c>
+      <c r="G49" s="46" t="inlineStr">
+        <is>
+          <t>kg 1,4-DCB</t>
+        </is>
+      </c>
+      <c r="H49" s="48" t="n">
+        <v>0.04657769823663591</v>
+      </c>
+      <c r="I49" s="48" t="n">
+        <v>0.723739548078785</v>
+      </c>
+    </row>
+    <row r="50" ht="36" customHeight="1">
+      <c r="B50" s="44" t="n">
+        <v>8</v>
+      </c>
+      <c r="C50" s="44" t="inlineStr">
+        <is>
+          <t>ETP Marine — Ecotoxicity — Marine</t>
+        </is>
+      </c>
+      <c r="D50" s="45" t="inlineStr">
+        <is>
+          <t>5. Overburden Removal
+Diesel {RoW}| diesel production, petroleum refinery operation | Cut-off, S</t>
+        </is>
+      </c>
+      <c r="E50" s="46" t="inlineStr">
+        <is>
+          <t>Nickel
+[Air]</t>
+        </is>
+      </c>
+      <c r="F50" s="47" t="n">
+        <v>0.00070836643</v>
+      </c>
+      <c r="G50" s="46" t="inlineStr">
+        <is>
+          <t>kg 1,4-DCB</t>
+        </is>
+      </c>
+      <c r="H50" s="48" t="n">
+        <v>0.02971187261575984</v>
+      </c>
+      <c r="I50" s="48" t="n">
+        <v>0.7534514206945448</v>
+      </c>
+    </row>
+    <row r="51" ht="36" customHeight="1">
+      <c r="B51" s="44" t="n">
+        <v>9</v>
+      </c>
+      <c r="C51" s="44" t="inlineStr">
+        <is>
+          <t>ETP Marine — Ecotoxicity — Marine</t>
+        </is>
+      </c>
+      <c r="D51" s="45" t="inlineStr">
+        <is>
+          <t>5. Overburden Removal
+Diesel {RoW}| diesel production, petroleum refinery operation | Cut-off, S</t>
+        </is>
+      </c>
+      <c r="E51" s="46" t="inlineStr">
+        <is>
+          <t>Barium
+[Water]</t>
+        </is>
+      </c>
+      <c r="F51" s="47" t="n">
+        <v>0.00063260735</v>
+      </c>
+      <c r="G51" s="46" t="inlineStr">
+        <is>
+          <t>kg 1,4-DCB</t>
+        </is>
+      </c>
+      <c r="H51" s="48" t="n">
+        <v>0.02653421760683013</v>
+      </c>
+      <c r="I51" s="48" t="n">
+        <v>0.779985638301375</v>
+      </c>
+    </row>
+    <row r="52" ht="36" customHeight="1">
+      <c r="B52" s="44" t="n">
+        <v>10</v>
+      </c>
+      <c r="C52" s="44" t="inlineStr">
+        <is>
+          <t>ETP Marine — Ecotoxicity — Marine</t>
+        </is>
+      </c>
+      <c r="D52" s="45" t="inlineStr">
+        <is>
+          <t>1. Supporting Material Production and Transportation
+Ammonium nitrate {RoW}| market for ammonium nitrate | Cut-off, S</t>
+        </is>
+      </c>
+      <c r="E52" s="46" t="inlineStr">
+        <is>
+          <t>Chlorpyrifos
+[Soil]</t>
+        </is>
+      </c>
+      <c r="F52" s="47" t="n">
+        <v>0.00049416215</v>
+      </c>
+      <c r="G52" s="46" t="inlineStr">
+        <is>
+          <t>kg 1,4-DCB</t>
+        </is>
+      </c>
+      <c r="H52" s="48" t="n">
+        <v>0.0207272426113276</v>
+      </c>
+      <c r="I52" s="48" t="n">
+        <v>0.8007128809127027</v>
+      </c>
+    </row>
+    <row r="53" ht="36" customHeight="1">
+      <c r="B53" s="44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C53" s="44" t="inlineStr">
+        <is>
+          <t>HTC — Human toxicity (karsinogenik)</t>
+        </is>
+      </c>
+      <c r="D53" s="45" t="inlineStr">
+        <is>
+          <t>5. Overburden Removal
+Palm oil, crude {MY}| palm oil mill operation | Cut-off, S</t>
+        </is>
+      </c>
+      <c r="E53" s="46" t="inlineStr">
+        <is>
+          <t>Chromium VI
+[Water]</t>
+        </is>
+      </c>
+      <c r="F53" s="47" t="n">
+        <v>0.022563787</v>
+      </c>
+      <c r="G53" s="46" t="inlineStr">
+        <is>
+          <t>kg 1,4-DCB</t>
+        </is>
+      </c>
+      <c r="H53" s="48" t="n">
+        <v>0.444150972127787</v>
+      </c>
+      <c r="I53" s="48" t="n">
+        <v>0.444150972127787</v>
+      </c>
+    </row>
+    <row r="54" ht="36" customHeight="1">
+      <c r="B54" s="44" t="n">
+        <v>2</v>
+      </c>
+      <c r="C54" s="44" t="inlineStr">
+        <is>
+          <t>HTC — Human toxicity (karsinogenik)</t>
+        </is>
+      </c>
+      <c r="D54" s="45" t="inlineStr">
+        <is>
+          <t>1. Supporting Material Production and Transportation
+Ammonium nitrate {RoW}| market for ammonium nitrate | Cut-off, S</t>
+        </is>
+      </c>
+      <c r="E54" s="46" t="inlineStr">
+        <is>
+          <t>Chromium VI
+[Water]</t>
+        </is>
+      </c>
+      <c r="F54" s="47" t="n">
+        <v>0.015112259</v>
+      </c>
+      <c r="G54" s="46" t="inlineStr">
+        <is>
+          <t>kg 1,4-DCB</t>
+        </is>
+      </c>
+      <c r="H54" s="48" t="n">
+        <v>0.2974733153568991</v>
+      </c>
+      <c r="I54" s="48" t="n">
+        <v>0.7416242874846861</v>
+      </c>
+    </row>
+    <row r="55" ht="36" customHeight="1">
+      <c r="B55" s="44" t="n">
+        <v>3</v>
+      </c>
+      <c r="C55" s="44" t="inlineStr">
+        <is>
+          <t>HTC — Human toxicity (karsinogenik)</t>
+        </is>
+      </c>
+      <c r="D55" s="45" t="inlineStr">
+        <is>
+          <t>5. Overburden Removal
+Palm oil, crude {MY}| palm oil mill operation | Cut-off, S</t>
+        </is>
+      </c>
+      <c r="E55" s="46" t="inlineStr">
+        <is>
+          <t>Furan
+[Air]</t>
+        </is>
+      </c>
+      <c r="F55" s="47" t="n">
+        <v>0.0028673737</v>
+      </c>
+      <c r="G55" s="46" t="inlineStr">
+        <is>
+          <t>kg 1,4-DCB</t>
+        </is>
+      </c>
+      <c r="H55" s="48" t="n">
+        <v>0.05644206871429205</v>
+      </c>
+      <c r="I55" s="48" t="n">
+        <v>0.7980663561989781</v>
+      </c>
+    </row>
+    <row r="56" ht="36" customHeight="1">
+      <c r="B56" s="44" t="n">
+        <v>4</v>
+      </c>
+      <c r="C56" s="44" t="inlineStr">
+        <is>
+          <t>HTC — Human toxicity (karsinogenik)</t>
+        </is>
+      </c>
+      <c r="D56" s="45" t="inlineStr">
+        <is>
+          <t>5. Overburden Removal
+Palm oil, crude {MY}| palm oil mill operation | Cut-off, S</t>
+        </is>
+      </c>
+      <c r="E56" s="46" t="inlineStr">
+        <is>
+          <t>Nickel
+[Air]</t>
+        </is>
+      </c>
+      <c r="F56" s="47" t="n">
+        <v>0.0024840857</v>
+      </c>
+      <c r="G56" s="46" t="inlineStr">
+        <is>
+          <t>kg 1,4-DCB</t>
+        </is>
+      </c>
+      <c r="H56" s="48" t="n">
+        <v>0.04889733618313869</v>
+      </c>
+      <c r="I56" s="48" t="n">
+        <v>0.8469636923821169</v>
+      </c>
+    </row>
+    <row r="57" ht="36" customHeight="1">
+      <c r="B57" s="44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C57" s="44" t="inlineStr">
+        <is>
+          <t>HTN — Human toxicity (non-karsinogenik)</t>
+        </is>
+      </c>
+      <c r="D57" s="45" t="inlineStr">
+        <is>
+          <t>1. Supporting Material Production and Transportation
+Ammonium nitrate {RoW}| market for ammonium nitrate | Cut-off, S</t>
+        </is>
+      </c>
+      <c r="E57" s="46" t="inlineStr">
+        <is>
+          <t>Arsenic
+[Water]</t>
+        </is>
+      </c>
+      <c r="F57" s="47" t="n">
+        <v>0.12820966</v>
+      </c>
+      <c r="G57" s="46" t="inlineStr">
+        <is>
+          <t>kg 1,4-DCB</t>
+        </is>
+      </c>
+      <c r="H57" s="48" t="n">
+        <v>0.3211400403979762</v>
+      </c>
+      <c r="I57" s="48" t="n">
+        <v>0.3211400403979762</v>
+      </c>
+    </row>
+    <row r="58" ht="36" customHeight="1">
+      <c r="B58" s="44" t="n">
+        <v>2</v>
+      </c>
+      <c r="C58" s="44" t="inlineStr">
+        <is>
+          <t>HTN — Human toxicity (non-karsinogenik)</t>
+        </is>
+      </c>
+      <c r="D58" s="45" t="inlineStr">
+        <is>
+          <t>5. Overburden Removal
+Diesel {RoW}| diesel production, petroleum refinery operation | Cut-off, S</t>
+        </is>
+      </c>
+      <c r="E58" s="46" t="inlineStr">
+        <is>
+          <t>Zinc
+[Water]</t>
+        </is>
+      </c>
+      <c r="F58" s="47" t="n">
+        <v>0.12050073</v>
+      </c>
+      <c r="G58" s="46" t="inlineStr">
+        <is>
+          <t>kg 1,4-DCB</t>
+        </is>
+      </c>
+      <c r="H58" s="48" t="n">
+        <v>0.30183068343045</v>
+      </c>
+      <c r="I58" s="48" t="n">
+        <v>0.6229707238284262</v>
+      </c>
+    </row>
+    <row r="59" ht="36" customHeight="1">
+      <c r="B59" s="44" t="n">
+        <v>3</v>
+      </c>
+      <c r="C59" s="44" t="inlineStr">
+        <is>
+          <t>HTN — Human toxicity (non-karsinogenik)</t>
+        </is>
+      </c>
+      <c r="D59" s="45" t="inlineStr">
+        <is>
+          <t>5. Overburden Removal
+Diesel {RoW}| diesel production, petroleum refinery operation | Cut-off, S</t>
+        </is>
+      </c>
+      <c r="E59" s="46" t="inlineStr">
+        <is>
+          <t>Arsenic
+[Water]</t>
+        </is>
+      </c>
+      <c r="F59" s="47" t="n">
+        <v>0.11253666</v>
+      </c>
+      <c r="G59" s="46" t="inlineStr">
+        <is>
+          <t>kg 1,4-DCB</t>
+        </is>
+      </c>
+      <c r="H59" s="48" t="n">
+        <v>0.2818822508276936</v>
+      </c>
+      <c r="I59" s="48" t="n">
+        <v>0.9048529746561198</v>
+      </c>
+    </row>
+    <row r="60" ht="36" customHeight="1">
+      <c r="B60" s="44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C60" s="44" t="inlineStr">
+        <is>
+          <t>WSF — Water scarcity footprint</t>
+        </is>
+      </c>
+      <c r="D60" s="45" t="inlineStr">
+        <is>
+          <t>1. Supporting Material Production and Transportation
+Textile, knit cotton {GLO}| market for | Cut-off, S</t>
+        </is>
+      </c>
+      <c r="E60" s="46" t="inlineStr">
+        <is>
+          <t>Water, turbine use, unspecified natural origin, RoW
+[Raw]</t>
+        </is>
+      </c>
+      <c r="F60" s="47" t="n">
+        <v>34.802798</v>
+      </c>
+      <c r="G60" s="46" t="inlineStr">
+        <is>
+          <t>m3</t>
+        </is>
+      </c>
+      <c r="H60" s="48" t="n">
+        <v>10.76044373244341</v>
+      </c>
+      <c r="I60" s="48" t="n">
+        <v>10.76044373244341</v>
+      </c>
+    </row>
+    <row r="61" ht="36" customHeight="1">
+      <c r="B61" s="44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C61" s="44" t="inlineStr">
+        <is>
+          <t>LUC — Land use change</t>
+        </is>
+      </c>
+      <c r="D61" s="45" t="inlineStr">
+        <is>
+          <t>2. Land Clearing
+2. Land Clearing</t>
+        </is>
+      </c>
+      <c r="E61" s="46" t="inlineStr">
+        <is>
+          <t>Transformation, from forest, intensive, ID
+[Raw]</t>
+        </is>
+      </c>
+      <c r="F61" s="47" t="n">
+        <v>8.547598199999999</v>
+      </c>
+      <c r="G61" s="46" t="inlineStr">
+        <is>
+          <t>m2a crop eq</t>
+        </is>
+      </c>
+      <c r="H61" s="48" t="n">
+        <v>0.6904020795745992</v>
+      </c>
+      <c r="I61" s="48" t="n">
+        <v>0.6904020795745992</v>
+      </c>
+    </row>
+    <row r="62" ht="36" customHeight="1">
+      <c r="B62" s="44" t="n">
+        <v>2</v>
+      </c>
+      <c r="C62" s="44" t="inlineStr">
+        <is>
+          <t>LUC — Land use change</t>
+        </is>
+      </c>
+      <c r="D62" s="45" t="inlineStr">
+        <is>
+          <t>5. Overburden Removal
+Palm oil, crude {MY}| palm oil mill operation | Cut-off, S</t>
+        </is>
+      </c>
+      <c r="E62" s="46" t="inlineStr">
+        <is>
+          <t>Occupation, permanent crop
+[Raw]</t>
+        </is>
+      </c>
+      <c r="F62" s="47" t="n">
+        <v>1.8451383</v>
+      </c>
+      <c r="G62" s="46" t="inlineStr">
+        <is>
+          <t>m2a crop eq</t>
+        </is>
+      </c>
+      <c r="H62" s="48" t="n">
+        <v>0.1490345345693415</v>
+      </c>
+      <c r="I62" s="48" t="n">
+        <v>0.8394366141439407</v>
+      </c>
+    </row>
+    <row r="63" ht="24" customHeight="1">
+      <c r="B63" s="41" t="inlineStr">
+        <is>
+          <t>Dampak Pemakaian Energi</t>
+        </is>
+      </c>
+      <c r="C63" s="42" t="n"/>
+      <c r="D63" s="42" t="n"/>
+      <c r="E63" s="42" t="n"/>
+      <c r="F63" s="42" t="n"/>
+      <c r="G63" s="42" t="n"/>
+      <c r="H63" s="42" t="n"/>
+      <c r="I63" s="43" t="n"/>
+    </row>
+    <row r="64" ht="36" customHeight="1">
+      <c r="B64" s="44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C64" s="44" t="inlineStr">
+        <is>
+          <t>CEN — Cumulative energy demand — non-renewable</t>
+        </is>
+      </c>
+      <c r="D64" s="45" t="inlineStr">
+        <is>
+          <t>5. Overburden Removal
+Diesel {RoW}| diesel production, petroleum refinery operation | Cut-off, S</t>
+        </is>
+      </c>
+      <c r="E64" s="46" t="inlineStr">
+        <is>
+          <t>Oil, crude
+[Raw]</t>
+        </is>
+      </c>
+      <c r="F64" s="47" t="n">
+        <v>139.10968</v>
+      </c>
+      <c r="G64" s="46" t="inlineStr">
+        <is>
+          <t>MJ</t>
+        </is>
+      </c>
+      <c r="H64" s="48" t="n">
+        <v>0.7516238188900974</v>
+      </c>
+      <c r="I64" s="48" t="n">
+        <v>0.7516238188900974</v>
+      </c>
+    </row>
+    <row r="65" ht="36" customHeight="1">
+      <c r="B65" s="44" t="n">
+        <v>2</v>
+      </c>
+      <c r="C65" s="44" t="inlineStr">
+        <is>
+          <t>CEN — Cumulative energy demand — non-renewable</t>
+        </is>
+      </c>
+      <c r="D65" s="45" t="inlineStr">
+        <is>
+          <t>5. Overburden Removal
+Diesel {RoW}| diesel production, petroleum refinery operation | Cut-off, S</t>
+        </is>
+      </c>
+      <c r="E65" s="46" t="inlineStr">
+        <is>
+          <t>Gas, natural/m3
+[Raw]</t>
+        </is>
+      </c>
+      <c r="F65" s="47" t="n">
+        <v>12.02628</v>
+      </c>
+      <c r="G65" s="46" t="inlineStr">
+        <is>
+          <t>MJ</t>
+        </is>
+      </c>
+      <c r="H65" s="48" t="n">
+        <v>0.06497921999850478</v>
+      </c>
+      <c r="I65" s="48" t="n">
+        <v>0.8166030388886022</v>
+      </c>
+    </row>
+    <row r="66" ht="36" customHeight="1">
+      <c r="B66" s="44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C66" s="44" t="inlineStr">
+        <is>
+          <t>CED — Cumulative energy demand — renewable</t>
+        </is>
+      </c>
+      <c r="D66" s="45" t="inlineStr">
+        <is>
+          <t>5. Overburden Removal
+Palm oil, crude {MY}| palm oil mill operation | Cut-off, S</t>
+        </is>
+      </c>
+      <c r="E66" s="46" t="inlineStr">
+        <is>
+          <t>Energy, gross calorific value, in biomass
+[Raw]</t>
+        </is>
+      </c>
+      <c r="F66" s="47" t="n">
+        <v>121.67912</v>
+      </c>
+      <c r="G66" s="46" t="inlineStr">
+        <is>
+          <t>MJ</t>
+        </is>
+      </c>
+      <c r="H66" s="48" t="n">
+        <v>0.9599700258710046</v>
+      </c>
+      <c r="I66" s="48" t="n">
+        <v>0.9599700258710046</v>
+      </c>
+    </row>
+    <row r="68" ht="35" customHeight="1">
+      <c r="B68" s="49" t="inlineStr">
+        <is>
+          <t>* Proses terkait ialah proses dengan kontribusi terbesar pada kategori dan unit yang sama di sheet PROC; data LCI tidak mengaitkan inventori langsung ke proses individual.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="25" customHeight="1">
+      <c r="B69" s="50" t="inlineStr">
+        <is>
+          <t>Sumber: SimaPro LMO.xlsx / LCI HULU LMO. Nilai dihitung dari tabel kanan; kontribusi bertanda = nilai / |total|. CEN/CED diagregasi; ETP terpisah.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="14">
+    <mergeCell ref="I5:I7"/>
+    <mergeCell ref="B18:I18"/>
+    <mergeCell ref="B68:I68"/>
+    <mergeCell ref="D5:D7"/>
+    <mergeCell ref="B69:I69"/>
+    <mergeCell ref="B2:I3"/>
+    <mergeCell ref="C5:C7"/>
+    <mergeCell ref="G5:G7"/>
+    <mergeCell ref="E5:E7"/>
+    <mergeCell ref="B63:I63"/>
+    <mergeCell ref="H5:H7"/>
+    <mergeCell ref="F5:F7"/>
+    <mergeCell ref="B8:I8"/>
+    <mergeCell ref="B5:B7"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="B2:I87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1013,7 +3215,7 @@
       </c>
       <c r="D5" s="22" t="inlineStr">
         <is>
-          <t>Unit proses / proses terkait*</t>
+          <t>Unit proses / proses terkait (bukan asal inventori)*</t>
         </is>
       </c>
       <c r="E5" s="22" t="inlineStr">
@@ -3804,7 +6006,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3861,7 +6063,7 @@
       </c>
       <c r="D5" s="22" t="inlineStr">
         <is>
-          <t>Unit proses / proses terkait*</t>
+          <t>Unit proses / proses terkait (bukan asal inventori)*</t>
         </is>
       </c>
       <c r="E5" s="22" t="inlineStr">

</xml_diff>